<commit_message>
fix weeks' number in timeline
</commit_message>
<xml_diff>
--- a/plan/v2.0/Anti_Scam_Weekly_Task_Tracker_2026_2027.xlsx
+++ b/plan/v2.0/Anti_Scam_Weekly_Task_Tracker_2026_2027.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb914ef0abe1a45e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Roadmap" sheetId="2" r:id="R08c2aca1d679490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Tracker" sheetId="3" r:id="R33a905f734fe4879"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Calendar" sheetId="4" r:id="R6b23ff84941d443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 tuần đầu" sheetId="5" r:id="R653f580b35da4944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WP Catalog" sheetId="6" r:id="Rc16e3f8b3d2b40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meetings &amp; Reports" sheetId="7" r:id="R6bc2f8e2b48c4fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R94d8f6ee7aab4f70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Roadmap" sheetId="2" r:id="Ra13062311daf44de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Tracker" sheetId="3" r:id="R7def9a2d6741400e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Calendar" sheetId="4" r:id="R3ef2fe38e6cb4c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 tuần đầu" sheetId="5" r:id="Rf7f973dcf270471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WP Catalog" sheetId="6" r:id="Rf6605c2482ef4299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meetings &amp; Reports" sheetId="7" r:id="R560d6875b7aa49ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -165,14 +165,14 @@
         <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -556,7 +556,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22" t="str">
-        <x:v>Release gate: CI baseline từ B0; CD/migration/image pipeline hoàn tất trước 20/10; 27–30/10 freeze/regression/release.</x:v>
+        <x:v>Release gate: CI baseline từ W09; CD/migration/image pipeline hoàn tất trước 20/10; 27–30/10 freeze/regression/release.</x:v>
       </x:c>
       <x:c r="B10" s="22"/>
       <x:c r="C10" s="22"/>
@@ -878,7 +878,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W09</x:v>
       </x:c>
       <x:c r="B2" s="28" t="n">
         <x:v>46292</x:v>
@@ -931,7 +931,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W09</x:v>
       </x:c>
       <x:c r="B3" s="28" t="n">
         <x:v>46292</x:v>
@@ -984,7 +984,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W09</x:v>
       </x:c>
       <x:c r="B4" s="28" t="n">
         <x:v>46292</x:v>
@@ -1037,7 +1037,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W09</x:v>
       </x:c>
       <x:c r="B5" s="28" t="n">
         <x:v>46292</x:v>
@@ -1090,7 +1090,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W09</x:v>
       </x:c>
       <x:c r="B6" s="28" t="n">
         <x:v>46292</x:v>
@@ -1143,7 +1143,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B7" s="28" t="n">
         <x:v>46301</x:v>
@@ -1196,7 +1196,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:v>46301</x:v>
@@ -1249,7 +1249,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B9" s="28" t="n">
         <x:v>46301</x:v>
@@ -1302,7 +1302,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:v>46301</x:v>
@@ -1355,7 +1355,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B11" s="28" t="n">
         <x:v>46301</x:v>
@@ -1408,7 +1408,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B12" s="28" t="n">
         <x:v>46308</x:v>
@@ -1461,7 +1461,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B13" s="28" t="n">
         <x:v>46308</x:v>
@@ -1514,7 +1514,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B14" s="28" t="n">
         <x:v>46308</x:v>
@@ -1567,7 +1567,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B15" s="28" t="n">
         <x:v>46308</x:v>
@@ -1620,7 +1620,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B16" s="28" t="n">
         <x:v>46308</x:v>
@@ -1673,7 +1673,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B17" s="28" t="n">
         <x:v>46308</x:v>
@@ -1726,7 +1726,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B18" s="28" t="n">
         <x:v>46315</x:v>
@@ -1779,7 +1779,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B19" s="28" t="n">
         <x:v>46315</x:v>
@@ -1832,7 +1832,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B20" s="28" t="n">
         <x:v>46315</x:v>
@@ -1885,7 +1885,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B21" s="28" t="n">
         <x:v>46315</x:v>
@@ -1938,7 +1938,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B22" s="28" t="n">
         <x:v>46315</x:v>
@@ -1991,7 +1991,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B23" s="28" t="n">
         <x:v>46315</x:v>
@@ -2044,7 +2044,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B24" s="28" t="n">
         <x:v>46322</x:v>
@@ -2097,7 +2097,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B25" s="28" t="n">
         <x:v>46322</x:v>
@@ -2150,7 +2150,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B26" s="28" t="n">
         <x:v>46322</x:v>
@@ -2203,7 +2203,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B27" s="28" t="n">
         <x:v>46322</x:v>
@@ -2256,7 +2256,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B28" s="28" t="n">
         <x:v>46322</x:v>
@@ -2309,7 +2309,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B29" s="28" t="n">
         <x:v>46322</x:v>
@@ -2362,7 +2362,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="27" t="str">
-        <x:v>W05</x:v>
+        <x:v>W14</x:v>
       </x:c>
       <x:c r="B30" s="28" t="n">
         <x:v>46329</x:v>
@@ -2415,7 +2415,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="27" t="str">
-        <x:v>W05</x:v>
+        <x:v>W14</x:v>
       </x:c>
       <x:c r="B31" s="28" t="n">
         <x:v>46329</x:v>
@@ -2468,7 +2468,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="27" t="str">
-        <x:v>W05</x:v>
+        <x:v>W14</x:v>
       </x:c>
       <x:c r="B32" s="28" t="n">
         <x:v>46329</x:v>
@@ -2521,7 +2521,7 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="27" t="str">
-        <x:v>W05</x:v>
+        <x:v>W14</x:v>
       </x:c>
       <x:c r="B33" s="28" t="n">
         <x:v>46329</x:v>
@@ -2574,7 +2574,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="27" t="str">
-        <x:v>W06</x:v>
+        <x:v>W15</x:v>
       </x:c>
       <x:c r="B34" s="28" t="n">
         <x:v>46336</x:v>
@@ -2627,7 +2627,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="27" t="str">
-        <x:v>W06</x:v>
+        <x:v>W15</x:v>
       </x:c>
       <x:c r="B35" s="28" t="n">
         <x:v>46336</x:v>
@@ -2680,7 +2680,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="27" t="str">
-        <x:v>W06</x:v>
+        <x:v>W15</x:v>
       </x:c>
       <x:c r="B36" s="28" t="n">
         <x:v>46336</x:v>
@@ -2733,7 +2733,7 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="27" t="str">
-        <x:v>W06</x:v>
+        <x:v>W15</x:v>
       </x:c>
       <x:c r="B37" s="28" t="n">
         <x:v>46336</x:v>
@@ -2786,7 +2786,7 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="27" t="str">
-        <x:v>W07</x:v>
+        <x:v>W16</x:v>
       </x:c>
       <x:c r="B38" s="28" t="n">
         <x:v>46343</x:v>
@@ -2839,7 +2839,7 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="27" t="str">
-        <x:v>W07</x:v>
+        <x:v>W16</x:v>
       </x:c>
       <x:c r="B39" s="28" t="n">
         <x:v>46343</x:v>
@@ -2892,7 +2892,7 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="27" t="str">
-        <x:v>W07</x:v>
+        <x:v>W16</x:v>
       </x:c>
       <x:c r="B40" s="28" t="n">
         <x:v>46343</x:v>
@@ -2945,7 +2945,7 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="27" t="str">
-        <x:v>W07</x:v>
+        <x:v>W16</x:v>
       </x:c>
       <x:c r="B41" s="28" t="n">
         <x:v>46343</x:v>
@@ -2998,7 +2998,7 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="27" t="str">
-        <x:v>W08</x:v>
+        <x:v>W17</x:v>
       </x:c>
       <x:c r="B42" s="28" t="n">
         <x:v>46350</x:v>
@@ -3051,7 +3051,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="27" t="str">
-        <x:v>W08</x:v>
+        <x:v>W17</x:v>
       </x:c>
       <x:c r="B43" s="28" t="n">
         <x:v>46350</x:v>
@@ -3104,7 +3104,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="27" t="str">
-        <x:v>W08</x:v>
+        <x:v>W17</x:v>
       </x:c>
       <x:c r="B44" s="28" t="n">
         <x:v>46350</x:v>
@@ -3157,7 +3157,7 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="27" t="str">
-        <x:v>W08</x:v>
+        <x:v>W17</x:v>
       </x:c>
       <x:c r="B45" s="28" t="n">
         <x:v>46350</x:v>
@@ -3210,7 +3210,7 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="27" t="str">
-        <x:v>W09</x:v>
+        <x:v>W18</x:v>
       </x:c>
       <x:c r="B46" s="28" t="n">
         <x:v>46357</x:v>
@@ -3263,7 +3263,7 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="27" t="str">
-        <x:v>W09</x:v>
+        <x:v>W18</x:v>
       </x:c>
       <x:c r="B47" s="28" t="n">
         <x:v>46357</x:v>
@@ -3316,7 +3316,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="27" t="str">
-        <x:v>W09</x:v>
+        <x:v>W18</x:v>
       </x:c>
       <x:c r="B48" s="28" t="n">
         <x:v>46357</x:v>
@@ -3369,7 +3369,7 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="27" t="str">
-        <x:v>W09</x:v>
+        <x:v>W18</x:v>
       </x:c>
       <x:c r="B49" s="28" t="n">
         <x:v>46357</x:v>
@@ -3422,7 +3422,7 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="27" t="str">
-        <x:v>W10</x:v>
+        <x:v>W19</x:v>
       </x:c>
       <x:c r="B50" s="28" t="n">
         <x:v>46364</x:v>
@@ -3475,7 +3475,7 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="27" t="str">
-        <x:v>W10</x:v>
+        <x:v>W19</x:v>
       </x:c>
       <x:c r="B51" s="28" t="n">
         <x:v>46364</x:v>
@@ -3528,7 +3528,7 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="27" t="str">
-        <x:v>W10</x:v>
+        <x:v>W19</x:v>
       </x:c>
       <x:c r="B52" s="28" t="n">
         <x:v>46364</x:v>
@@ -3581,7 +3581,7 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="27" t="str">
-        <x:v>W11</x:v>
+        <x:v>W20</x:v>
       </x:c>
       <x:c r="B53" s="28" t="n">
         <x:v>46371</x:v>
@@ -3634,7 +3634,7 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="27" t="str">
-        <x:v>W11</x:v>
+        <x:v>W20</x:v>
       </x:c>
       <x:c r="B54" s="28" t="n">
         <x:v>46371</x:v>
@@ -3687,7 +3687,7 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="27" t="str">
-        <x:v>W11</x:v>
+        <x:v>W20</x:v>
       </x:c>
       <x:c r="B55" s="28" t="n">
         <x:v>46371</x:v>
@@ -3740,7 +3740,7 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="27" t="str">
-        <x:v>W14</x:v>
+        <x:v>W23</x:v>
       </x:c>
       <x:c r="B56" s="28" t="n">
         <x:v>46392</x:v>
@@ -3793,7 +3793,7 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="27" t="str">
-        <x:v>W14</x:v>
+        <x:v>W23</x:v>
       </x:c>
       <x:c r="B57" s="28" t="n">
         <x:v>46392</x:v>
@@ -3846,7 +3846,7 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="27" t="str">
-        <x:v>W14</x:v>
+        <x:v>W23</x:v>
       </x:c>
       <x:c r="B58" s="28" t="n">
         <x:v>46392</x:v>
@@ -3899,7 +3899,7 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="27" t="str">
-        <x:v>W15</x:v>
+        <x:v>W24</x:v>
       </x:c>
       <x:c r="B59" s="28" t="n">
         <x:v>46399</x:v>
@@ -3952,7 +3952,7 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="27" t="str">
-        <x:v>W15</x:v>
+        <x:v>W24</x:v>
       </x:c>
       <x:c r="B60" s="28" t="n">
         <x:v>46399</x:v>
@@ -4005,7 +4005,7 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="27" t="str">
-        <x:v>W15</x:v>
+        <x:v>W24</x:v>
       </x:c>
       <x:c r="B61" s="28" t="n">
         <x:v>46399</x:v>
@@ -4058,7 +4058,7 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="27" t="str">
-        <x:v>W20</x:v>
+        <x:v>W29</x:v>
       </x:c>
       <x:c r="B62" s="28" t="n">
         <x:v>46434</x:v>
@@ -4111,7 +4111,7 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="27" t="str">
-        <x:v>W20</x:v>
+        <x:v>W29</x:v>
       </x:c>
       <x:c r="B63" s="28" t="n">
         <x:v>46434</x:v>
@@ -4164,7 +4164,7 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="27" t="str">
-        <x:v>W21</x:v>
+        <x:v>W30</x:v>
       </x:c>
       <x:c r="B64" s="28" t="n">
         <x:v>46441</x:v>
@@ -4217,7 +4217,7 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="27" t="str">
-        <x:v>W21</x:v>
+        <x:v>W30</x:v>
       </x:c>
       <x:c r="B65" s="28" t="n">
         <x:v>46441</x:v>
@@ -4270,7 +4270,7 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="27" t="str">
-        <x:v>W22</x:v>
+        <x:v>W31</x:v>
       </x:c>
       <x:c r="B66" s="28" t="n">
         <x:v>46448</x:v>
@@ -4323,7 +4323,7 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="27" t="str">
-        <x:v>W22</x:v>
+        <x:v>W31</x:v>
       </x:c>
       <x:c r="B67" s="28" t="n">
         <x:v>46448</x:v>
@@ -4376,7 +4376,7 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="27" t="str">
-        <x:v>W23</x:v>
+        <x:v>W32</x:v>
       </x:c>
       <x:c r="B68" s="28" t="n">
         <x:v>46455</x:v>
@@ -4429,7 +4429,7 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="27" t="str">
-        <x:v>W28</x:v>
+        <x:v>W37</x:v>
       </x:c>
       <x:c r="B69" s="28" t="n">
         <x:v>46490</x:v>
@@ -4482,7 +4482,7 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="27" t="str">
-        <x:v>W28</x:v>
+        <x:v>W37</x:v>
       </x:c>
       <x:c r="B70" s="28" t="n">
         <x:v>46490</x:v>
@@ -4535,7 +4535,7 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="27" t="str">
-        <x:v>W29</x:v>
+        <x:v>W38</x:v>
       </x:c>
       <x:c r="B71" s="28" t="n">
         <x:v>46497</x:v>
@@ -4588,7 +4588,7 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="27" t="str">
-        <x:v>W29</x:v>
+        <x:v>W38</x:v>
       </x:c>
       <x:c r="B72" s="28" t="n">
         <x:v>46497</x:v>
@@ -4641,7 +4641,7 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="27" t="str">
-        <x:v>W31</x:v>
+        <x:v>W40</x:v>
       </x:c>
       <x:c r="B73" s="28" t="n">
         <x:v>46511</x:v>
@@ -4694,7 +4694,7 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="27" t="str">
-        <x:v>W32</x:v>
+        <x:v>W41</x:v>
       </x:c>
       <x:c r="B74" s="28" t="n">
         <x:v>46518</x:v>
@@ -4747,7 +4747,7 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="27" t="str">
-        <x:v>W33</x:v>
+        <x:v>W42</x:v>
       </x:c>
       <x:c r="B75" s="28" t="n">
         <x:v>46525</x:v>
@@ -4800,7 +4800,7 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="27" t="str">
-        <x:v>W33</x:v>
+        <x:v>W42</x:v>
       </x:c>
       <x:c r="B76" s="28" t="n">
         <x:v>46525</x:v>
@@ -4875,7 +4875,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5510aa17d7074a62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4c2c4da4a1f4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4946,7 +4946,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W09</x:v>
       </x:c>
       <x:c r="B2" s="28" t="n">
         <x:v>46292</x:v>
@@ -4990,7 +4990,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B3" s="28" t="n">
         <x:v>46301</x:v>
@@ -5034,7 +5034,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B4" s="28" t="n">
         <x:v>46308</x:v>
@@ -5078,7 +5078,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B5" s="28" t="n">
         <x:v>46315</x:v>
@@ -5122,7 +5122,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B6" s="28" t="n">
         <x:v>46322</x:v>
@@ -5166,7 +5166,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
-        <x:v>W05</x:v>
+        <x:v>W14</x:v>
       </x:c>
       <x:c r="B7" s="28" t="n">
         <x:v>46329</x:v>
@@ -5210,7 +5210,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="27" t="str">
-        <x:v>W06</x:v>
+        <x:v>W15</x:v>
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:v>46336</x:v>
@@ -5254,7 +5254,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="27" t="str">
-        <x:v>W07</x:v>
+        <x:v>W16</x:v>
       </x:c>
       <x:c r="B9" s="28" t="n">
         <x:v>46343</x:v>
@@ -5298,7 +5298,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27" t="str">
-        <x:v>W08</x:v>
+        <x:v>W17</x:v>
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:v>46350</x:v>
@@ -5342,7 +5342,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="27" t="str">
-        <x:v>W09</x:v>
+        <x:v>W18</x:v>
       </x:c>
       <x:c r="B11" s="28" t="n">
         <x:v>46357</x:v>
@@ -5386,7 +5386,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="27" t="str">
-        <x:v>W10</x:v>
+        <x:v>W19</x:v>
       </x:c>
       <x:c r="B12" s="28" t="n">
         <x:v>46364</x:v>
@@ -5430,7 +5430,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="27" t="str">
-        <x:v>W11</x:v>
+        <x:v>W20</x:v>
       </x:c>
       <x:c r="B13" s="28" t="n">
         <x:v>46371</x:v>
@@ -5474,7 +5474,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="27" t="str">
-        <x:v>W12</x:v>
+        <x:v>W21</x:v>
       </x:c>
       <x:c r="B14" s="28" t="n">
         <x:v>46378</x:v>
@@ -5518,7 +5518,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="27" t="str">
-        <x:v>W13</x:v>
+        <x:v>W22</x:v>
       </x:c>
       <x:c r="B15" s="28" t="n">
         <x:v>46385</x:v>
@@ -5562,7 +5562,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="27" t="str">
-        <x:v>W14</x:v>
+        <x:v>W23</x:v>
       </x:c>
       <x:c r="B16" s="28" t="n">
         <x:v>46392</x:v>
@@ -5606,7 +5606,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="27" t="str">
-        <x:v>W15</x:v>
+        <x:v>W24</x:v>
       </x:c>
       <x:c r="B17" s="28" t="n">
         <x:v>46399</x:v>
@@ -5650,7 +5650,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="27" t="str">
-        <x:v>W16</x:v>
+        <x:v>W25</x:v>
       </x:c>
       <x:c r="B18" s="28" t="n">
         <x:v>46406</x:v>
@@ -5694,7 +5694,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="27" t="str">
-        <x:v>W17</x:v>
+        <x:v>W26</x:v>
       </x:c>
       <x:c r="B19" s="28" t="n">
         <x:v>46413</x:v>
@@ -5738,7 +5738,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="27" t="str">
-        <x:v>W18</x:v>
+        <x:v>W27</x:v>
       </x:c>
       <x:c r="B20" s="28" t="n">
         <x:v>46420</x:v>
@@ -5782,7 +5782,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="27" t="str">
-        <x:v>W19</x:v>
+        <x:v>W28</x:v>
       </x:c>
       <x:c r="B21" s="28" t="n">
         <x:v>46427</x:v>
@@ -5826,7 +5826,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="27" t="str">
-        <x:v>W20</x:v>
+        <x:v>W29</x:v>
       </x:c>
       <x:c r="B22" s="28" t="n">
         <x:v>46434</x:v>
@@ -5870,7 +5870,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="27" t="str">
-        <x:v>W21</x:v>
+        <x:v>W30</x:v>
       </x:c>
       <x:c r="B23" s="28" t="n">
         <x:v>46441</x:v>
@@ -5914,7 +5914,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="27" t="str">
-        <x:v>W22</x:v>
+        <x:v>W31</x:v>
       </x:c>
       <x:c r="B24" s="28" t="n">
         <x:v>46448</x:v>
@@ -5958,7 +5958,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="27" t="str">
-        <x:v>W23</x:v>
+        <x:v>W32</x:v>
       </x:c>
       <x:c r="B25" s="28" t="n">
         <x:v>46455</x:v>
@@ -6002,7 +6002,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="27" t="str">
-        <x:v>W24</x:v>
+        <x:v>W33</x:v>
       </x:c>
       <x:c r="B26" s="28" t="n">
         <x:v>46462</x:v>
@@ -6046,7 +6046,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="27" t="str">
-        <x:v>W25</x:v>
+        <x:v>W34</x:v>
       </x:c>
       <x:c r="B27" s="28" t="n">
         <x:v>46469</x:v>
@@ -6090,7 +6090,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="27" t="str">
-        <x:v>W26</x:v>
+        <x:v>W35</x:v>
       </x:c>
       <x:c r="B28" s="28" t="n">
         <x:v>46476</x:v>
@@ -6134,7 +6134,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="27" t="str">
-        <x:v>W27</x:v>
+        <x:v>W36</x:v>
       </x:c>
       <x:c r="B29" s="28" t="n">
         <x:v>46483</x:v>
@@ -6178,7 +6178,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="27" t="str">
-        <x:v>W28</x:v>
+        <x:v>W37</x:v>
       </x:c>
       <x:c r="B30" s="28" t="n">
         <x:v>46490</x:v>
@@ -6222,7 +6222,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="27" t="str">
-        <x:v>W29</x:v>
+        <x:v>W38</x:v>
       </x:c>
       <x:c r="B31" s="28" t="n">
         <x:v>46497</x:v>
@@ -6266,7 +6266,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="27" t="str">
-        <x:v>W30</x:v>
+        <x:v>W39</x:v>
       </x:c>
       <x:c r="B32" s="28" t="n">
         <x:v>46504</x:v>
@@ -6310,7 +6310,7 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="27" t="str">
-        <x:v>W31</x:v>
+        <x:v>W40</x:v>
       </x:c>
       <x:c r="B33" s="28" t="n">
         <x:v>46511</x:v>
@@ -6354,7 +6354,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="27" t="str">
-        <x:v>W32</x:v>
+        <x:v>W41</x:v>
       </x:c>
       <x:c r="B34" s="28" t="n">
         <x:v>46518</x:v>
@@ -6398,7 +6398,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="27" t="str">
-        <x:v>W33</x:v>
+        <x:v>W42</x:v>
       </x:c>
       <x:c r="B35" s="28" t="n">
         <x:v>46525</x:v>
@@ -6442,7 +6442,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="27" t="str">
-        <x:v>W34</x:v>
+        <x:v>W43</x:v>
       </x:c>
       <x:c r="B36" s="28" t="n">
         <x:v>46532</x:v>
@@ -6486,7 +6486,7 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="27" t="str">
-        <x:v>W35</x:v>
+        <x:v>W44</x:v>
       </x:c>
       <x:c r="B37" s="28" t="n">
         <x:v>46539</x:v>
@@ -6530,7 +6530,7 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="27" t="str">
-        <x:v>W36</x:v>
+        <x:v>W45</x:v>
       </x:c>
       <x:c r="B38" s="28" t="n">
         <x:v>46546</x:v>
@@ -6574,7 +6574,7 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="27" t="str">
-        <x:v>W37</x:v>
+        <x:v>W47</x:v>
       </x:c>
       <x:c r="B39" s="28" t="n">
         <x:v>46553</x:v>
@@ -6618,7 +6618,7 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="27" t="str">
-        <x:v>W38</x:v>
+        <x:v>W48</x:v>
       </x:c>
       <x:c r="B40" s="28" t="n">
         <x:v>46560</x:v>
@@ -6662,7 +6662,7 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="27" t="str">
-        <x:v>W39</x:v>
+        <x:v>W49</x:v>
       </x:c>
       <x:c r="B41" s="28" t="n">
         <x:v>46567</x:v>
@@ -6706,7 +6706,7 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="27" t="str">
-        <x:v>W40</x:v>
+        <x:v>W50</x:v>
       </x:c>
       <x:c r="B42" s="28" t="n">
         <x:v>46574</x:v>
@@ -6750,7 +6750,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="27" t="str">
-        <x:v>W41</x:v>
+        <x:v>W51</x:v>
       </x:c>
       <x:c r="B43" s="28" t="n">
         <x:v>46581</x:v>
@@ -6794,7 +6794,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="27" t="str">
-        <x:v>W42</x:v>
+        <x:v>W52</x:v>
       </x:c>
       <x:c r="B44" s="28" t="n">
         <x:v>46588</x:v>
@@ -6838,7 +6838,7 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="27" t="str">
-        <x:v>W43</x:v>
+        <x:v>W53</x:v>
       </x:c>
       <x:c r="B45" s="28" t="n">
         <x:v>46595</x:v>
@@ -6935,7 +6935,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B2" s="27" t="str">
         <x:v>27/09 → 05/10</x:v>
@@ -6965,7 +6965,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B3" s="27" t="str">
         <x:v>27/09 → 05/10</x:v>
@@ -6995,7 +6995,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B4" s="27" t="str">
         <x:v>27/09 → 05/10</x:v>
@@ -7027,7 +7027,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B5" s="27" t="str">
         <x:v>27/09 → 05/10</x:v>
@@ -7057,7 +7057,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B6" s="27" t="str">
         <x:v>27/09 → 05/10</x:v>
@@ -7087,7 +7087,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B7" s="27" t="str">
         <x:v>27/09 → 05/10</x:v>
@@ -7117,7 +7117,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B8" s="27" t="str">
         <x:v>06/10 → 12/10</x:v>
@@ -7147,7 +7147,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B9" s="27" t="str">
         <x:v>06/10 → 12/10</x:v>
@@ -7177,7 +7177,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B10" s="27" t="str">
         <x:v>06/10 → 12/10</x:v>
@@ -7207,7 +7207,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B11" s="27" t="str">
         <x:v>06/10 → 12/10</x:v>
@@ -7237,7 +7237,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B12" s="27" t="str">
         <x:v>06/10 → 12/10</x:v>
@@ -7267,7 +7267,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B13" s="27" t="str">
         <x:v>06/10 → 12/10</x:v>
@@ -10028,7 +10028,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="27" t="str">
-        <x:v>B0</x:v>
+        <x:v>W10</x:v>
       </x:c>
       <x:c r="B2" s="28" t="n">
         <x:v>46296</x:v>
@@ -10051,7 +10051,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>W01</x:v>
+        <x:v>W11</x:v>
       </x:c>
       <x:c r="B3" s="28" t="n">
         <x:v>46303</x:v>
@@ -10074,7 +10074,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="27" t="str">
-        <x:v>W02</x:v>
+        <x:v>W12</x:v>
       </x:c>
       <x:c r="B4" s="28" t="n">
         <x:v>46310</x:v>
@@ -10097,7 +10097,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="27" t="str">
-        <x:v>W03</x:v>
+        <x:v>W13</x:v>
       </x:c>
       <x:c r="B5" s="28" t="n">
         <x:v>46317</x:v>
@@ -10120,7 +10120,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="27" t="str">
-        <x:v>W04</x:v>
+        <x:v>W14</x:v>
       </x:c>
       <x:c r="B6" s="28" t="n">
         <x:v>46324</x:v>
@@ -10143,7 +10143,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="27" t="str">
-        <x:v>W05</x:v>
+        <x:v>W15</x:v>
       </x:c>
       <x:c r="B7" s="28" t="n">
         <x:v>46331</x:v>
@@ -10166,7 +10166,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="27" t="str">
-        <x:v>W06</x:v>
+        <x:v>W16</x:v>
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:v>46338</x:v>
@@ -10189,7 +10189,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="27" t="str">
-        <x:v>W07</x:v>
+        <x:v>W17</x:v>
       </x:c>
       <x:c r="B9" s="28" t="n">
         <x:v>46345</x:v>
@@ -10212,7 +10212,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27" t="str">
-        <x:v>W08</x:v>
+        <x:v>W18</x:v>
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:v>46352</x:v>
@@ -10235,7 +10235,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="27" t="str">
-        <x:v>W09</x:v>
+        <x:v>W19</x:v>
       </x:c>
       <x:c r="B11" s="28" t="n">
         <x:v>46359</x:v>
@@ -10258,7 +10258,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="27" t="str">
-        <x:v>W10</x:v>
+        <x:v>W20</x:v>
       </x:c>
       <x:c r="B12" s="28" t="n">
         <x:v>46366</x:v>
@@ -10281,7 +10281,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="27" t="str">
-        <x:v>W11</x:v>
+        <x:v>W21</x:v>
       </x:c>
       <x:c r="B13" s="28" t="n">
         <x:v>46373</x:v>
@@ -10304,7 +10304,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="27" t="str">
-        <x:v>W12</x:v>
+        <x:v>W22</x:v>
       </x:c>
       <x:c r="B14" s="28" t="n">
         <x:v>46380</x:v>
@@ -10327,7 +10327,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="27" t="str">
-        <x:v>W13</x:v>
+        <x:v>W23</x:v>
       </x:c>
       <x:c r="B15" s="28" t="n">
         <x:v>46387</x:v>
@@ -10350,7 +10350,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="27" t="str">
-        <x:v>W14</x:v>
+        <x:v>W24</x:v>
       </x:c>
       <x:c r="B16" s="28" t="n">
         <x:v>46394</x:v>
@@ -10373,7 +10373,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="27" t="str">
-        <x:v>W15</x:v>
+        <x:v>W25</x:v>
       </x:c>
       <x:c r="B17" s="28" t="n">
         <x:v>46401</x:v>
@@ -10396,7 +10396,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="27" t="str">
-        <x:v>W16</x:v>
+        <x:v>W26</x:v>
       </x:c>
       <x:c r="B18" s="28" t="n">
         <x:v>46408</x:v>
@@ -10419,7 +10419,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="27" t="str">
-        <x:v>W17</x:v>
+        <x:v>W27</x:v>
       </x:c>
       <x:c r="B19" s="28" t="n">
         <x:v>46415</x:v>
@@ -10442,7 +10442,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="27" t="str">
-        <x:v>W18</x:v>
+        <x:v>W28</x:v>
       </x:c>
       <x:c r="B20" s="28" t="n">
         <x:v>46422</x:v>
@@ -10465,7 +10465,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="27" t="str">
-        <x:v>W19</x:v>
+        <x:v>W29</x:v>
       </x:c>
       <x:c r="B21" s="28" t="n">
         <x:v>46429</x:v>
@@ -10488,7 +10488,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="27" t="str">
-        <x:v>W20</x:v>
+        <x:v>W30</x:v>
       </x:c>
       <x:c r="B22" s="28" t="n">
         <x:v>46436</x:v>
@@ -10511,7 +10511,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="27" t="str">
-        <x:v>W21</x:v>
+        <x:v>W31</x:v>
       </x:c>
       <x:c r="B23" s="28" t="n">
         <x:v>46443</x:v>
@@ -10534,7 +10534,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="27" t="str">
-        <x:v>W22</x:v>
+        <x:v>W32</x:v>
       </x:c>
       <x:c r="B24" s="28" t="n">
         <x:v>46450</x:v>
@@ -10557,7 +10557,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="27" t="str">
-        <x:v>W23</x:v>
+        <x:v>W33</x:v>
       </x:c>
       <x:c r="B25" s="28" t="n">
         <x:v>46457</x:v>
@@ -10580,7 +10580,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="27" t="str">
-        <x:v>W24</x:v>
+        <x:v>W34</x:v>
       </x:c>
       <x:c r="B26" s="28" t="n">
         <x:v>46464</x:v>
@@ -10603,7 +10603,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="27" t="str">
-        <x:v>W25</x:v>
+        <x:v>W35</x:v>
       </x:c>
       <x:c r="B27" s="28" t="n">
         <x:v>46471</x:v>
@@ -10626,7 +10626,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="27" t="str">
-        <x:v>W26</x:v>
+        <x:v>W36</x:v>
       </x:c>
       <x:c r="B28" s="28" t="n">
         <x:v>46478</x:v>
@@ -10649,7 +10649,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="27" t="str">
-        <x:v>W27</x:v>
+        <x:v>W37</x:v>
       </x:c>
       <x:c r="B29" s="28" t="n">
         <x:v>46485</x:v>
@@ -10672,7 +10672,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="27" t="str">
-        <x:v>W28</x:v>
+        <x:v>W38</x:v>
       </x:c>
       <x:c r="B30" s="28" t="n">
         <x:v>46492</x:v>
@@ -10695,7 +10695,7 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="27" t="str">
-        <x:v>W29</x:v>
+        <x:v>W39</x:v>
       </x:c>
       <x:c r="B31" s="28" t="n">
         <x:v>46499</x:v>
@@ -10718,7 +10718,7 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="27" t="str">
-        <x:v>W30</x:v>
+        <x:v>W40</x:v>
       </x:c>
       <x:c r="B32" s="28" t="n">
         <x:v>46506</x:v>
@@ -10741,7 +10741,7 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="27" t="str">
-        <x:v>W31</x:v>
+        <x:v>W41</x:v>
       </x:c>
       <x:c r="B33" s="28" t="n">
         <x:v>46513</x:v>
@@ -10764,7 +10764,7 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="27" t="str">
-        <x:v>W32</x:v>
+        <x:v>W42</x:v>
       </x:c>
       <x:c r="B34" s="28" t="n">
         <x:v>46520</x:v>
@@ -10787,7 +10787,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="27" t="str">
-        <x:v>W33</x:v>
+        <x:v>W43</x:v>
       </x:c>
       <x:c r="B35" s="28" t="n">
         <x:v>46527</x:v>
@@ -10810,7 +10810,7 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="27" t="str">
-        <x:v>W34</x:v>
+        <x:v>W44</x:v>
       </x:c>
       <x:c r="B36" s="28" t="n">
         <x:v>46534</x:v>
@@ -10833,7 +10833,7 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="27" t="str">
-        <x:v>W35</x:v>
+        <x:v>W45</x:v>
       </x:c>
       <x:c r="B37" s="28" t="n">
         <x:v>46541</x:v>
@@ -10856,7 +10856,7 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="27" t="str">
-        <x:v>W36</x:v>
+        <x:v>W46</x:v>
       </x:c>
       <x:c r="B38" s="28" t="n">
         <x:v>46548</x:v>
@@ -10879,7 +10879,7 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="27" t="str">
-        <x:v>W37</x:v>
+        <x:v>W47</x:v>
       </x:c>
       <x:c r="B39" s="28" t="n">
         <x:v>46555</x:v>
@@ -10902,7 +10902,7 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="27" t="str">
-        <x:v>W38</x:v>
+        <x:v>W48</x:v>
       </x:c>
       <x:c r="B40" s="28" t="n">
         <x:v>46562</x:v>
@@ -10925,7 +10925,7 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="27" t="str">
-        <x:v>W39</x:v>
+        <x:v>W49</x:v>
       </x:c>
       <x:c r="B41" s="28" t="n">
         <x:v>46569</x:v>
@@ -10948,7 +10948,7 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="27" t="str">
-        <x:v>W40</x:v>
+        <x:v>W50</x:v>
       </x:c>
       <x:c r="B42" s="28" t="n">
         <x:v>46576</x:v>
@@ -10971,7 +10971,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="27" t="str">
-        <x:v>W41</x:v>
+        <x:v>W51</x:v>
       </x:c>
       <x:c r="B43" s="28" t="n">
         <x:v>46583</x:v>
@@ -10994,7 +10994,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="27" t="str">
-        <x:v>W42</x:v>
+        <x:v>W52</x:v>
       </x:c>
       <x:c r="B44" s="28" t="n">
         <x:v>46590</x:v>
@@ -11017,7 +11017,7 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="27" t="str">
-        <x:v>W43</x:v>
+        <x:v>W53</x:v>
       </x:c>
       <x:c r="B45" s="28" t="n">
         <x:v>46597</x:v>

</xml_diff>